<commit_message>
Upgrade results last intervention
</commit_message>
<xml_diff>
--- a/02_Output/G-Form/Summary_results/Table_population_effects_summary.xlsx
+++ b/02_Output/G-Form/Summary_results/Table_population_effects_summary.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
   <si>
     <t xml:space="preserve">Exposure and scenario</t>
   </si>
@@ -210,6 +210,27 @@
   </si>
   <si>
     <t xml:space="preserve">-2.97 (-5.25; -0.47)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; 10 ppbv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.17 (5.97; 9.43)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">51209 (42609; 67335)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.0480 (1.0033; 1.0926)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.33 (0.02; 0.63)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.33 (-0.63; -0.02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.80 (-9.28; -0.31)</t>
   </si>
   <si>
     <t xml:space="preserve">&lt; 5 ppbv</t>
@@ -955,94 +976,117 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>8</v>
+      <c r="B15" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>13</v>
+      <c r="A16" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>87</v>
+      <c r="B18" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>